<commit_message>
v1.0.52: fix Process only differences filtering across all four strategies; XC 71, GB 22, AP 26 tests pass
Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_data/fixtures/ap/ap_fip_ZQ9_VALMSG.xlsx
+++ b/test_data/fixtures/ap/ap_fip_ZQ9_VALMSG.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1040,6 +1040,110 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>V900W</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Test method</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>AP_DIFF_YELLOW</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>V900W|AP_DIFF_YELLOW</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>CLS</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>V900W</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Test method</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>AP_DIFF_GREEN</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>V900W|AP_DIFF_GREEN</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>CLS</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>001</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>w</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>